<commit_message>
Split partner and country into separate columns
The source table packed both into one "계약상대(국가)" cell, which made
the country unusable for filtering or grouping. Two columns now, with
the odd rows flagged in 비고: the 중남미 4개국 deal names no partner,
동아에스티/인타스 is listed as 다국적제약사 rather than a country, and
the 대웅제약 Middle East deal covers six countries at once.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jf57MMhcbMyWGo6aDm1iwR
</commit_message>
<xml_diff>
--- a/output/k_bio_licensing_33deals.xlsx
+++ b/output/k_bio_licensing_33deals.xlsx
@@ -10,7 +10,7 @@
     <sheet name="기술수출 33건" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'기술수출 33건'!$A$2:$I$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'기술수출 33건'!$A$2:$J$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -107,7 +107,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -491,18 +491,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -530,30 +531,35 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>계약상대(국가)</t>
+          <t>계약상대</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>국가</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>제품/적응증/기술</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>계약규모(만달러)</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>계약규모(억원)</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>원문(계약규모)</t>
         </is>
@@ -575,24 +581,29 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>인타스 파마슈티컬스(인도)</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
+          <t>인타스 파마슈티컬스</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>인도</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>인간 히알루로니다제(ALT-B4)</t>
         </is>
       </c>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n">
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n">
         <v>1250</v>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>달러 금액 미표기</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>약 1,250억원</t>
         </is>
@@ -614,22 +625,27 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>MSD(미국)</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
+          <t>MSD</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>미국</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>고형암에 쓰는 CAR-NK 세포치료제 3종(공동개발)</t>
         </is>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="G4" s="5" t="n">
         <v>186600</v>
       </c>
-      <c r="G4" s="5" t="n">
+      <c r="H4" s="5" t="n">
         <v>20900</v>
       </c>
-      <c r="H4" s="4" t="inlineStr"/>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr"/>
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>약 2조 900억원 (약 18억 6,600만 달러)</t>
         </is>
@@ -651,22 +667,27 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>KG바이오(인도네시아)</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
+          <t>KG바이오</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>인도네시아</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>GX-17(코로나19 치료제와 면역항암제로 개발 중)</t>
         </is>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="G5" s="5" t="n">
         <v>110000</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="H5" s="5" t="n">
         <v>12000</v>
       </c>
-      <c r="H5" s="4" t="inlineStr"/>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>약 1조 2,000억원 (약 11억 달러)</t>
         </is>
@@ -688,24 +709,29 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>상해하이니(중국)</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
+          <t>상해하이니</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>위식도역류질환 치료 신약 '펙수프라잔'</t>
         </is>
       </c>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n">
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n">
         <v>3800</v>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>달러 금액 미표기</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>약 3,800억원</t>
         </is>
@@ -727,22 +753,27 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>3D메디슨(중국)</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
+          <t>3D메디슨</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>CD47 항체 항암신약후보 물질 'IMC-002'</t>
         </is>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="G7" s="5" t="n">
         <v>47050</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="H7" s="5" t="n">
         <v>5400</v>
       </c>
-      <c r="H7" s="4" t="inlineStr"/>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>약 5,400억원 (약 4억 7,050만 달러)</t>
         </is>
@@ -764,22 +795,27 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>치루제약(중국)</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
+          <t>치루제약</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>표적항암 항체치료제 / MUC1 타겟 암 치료용 항체 후보 약물-접합체(ADC) 'PAb001-ADC'</t>
         </is>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="G8" s="5" t="n">
         <v>53900</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="H8" s="5" t="n">
         <v>6340</v>
       </c>
-      <c r="H8" s="4" t="inlineStr"/>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr"/>
+      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>약 6,340억원 (약 5억 3,900만 달러)</t>
         </is>
@@ -801,18 +837,23 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>트랜스테라 바이오사이언스(중국)</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
+          <t>트랜스테라 바이오사이언스</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>자가면역질환 치료 후보물질 'LC510255'</t>
         </is>
       </c>
-      <c r="F9" s="5" t="n"/>
       <c r="G9" s="5" t="n"/>
-      <c r="H9" s="4" t="inlineStr"/>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="4" t="inlineStr"/>
+      <c r="J9" s="4" t="inlineStr">
         <is>
           <t>비공개</t>
         </is>
@@ -834,22 +875,27 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>AUM바이오사이언스(싱가포르)</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
+          <t>AUM바이오사이언스</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>싱가포르</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>표적항암제 후보물질 CHC2014</t>
         </is>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="G10" s="5" t="n">
         <v>17250</v>
       </c>
-      <c r="G10" s="5" t="n">
+      <c r="H10" s="5" t="n">
         <v>1934</v>
       </c>
-      <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr"/>
+      <c r="J10" s="4" t="inlineStr">
         <is>
           <t>약 1,934억원 (약 1억 7,250만 달러)</t>
         </is>
@@ -871,22 +917,27 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>뉴로가스트릭스(미국)</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
+          <t>뉴로가스트릭스</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>미국</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>'펙수프라잔' 위식도역류질환 치료제</t>
         </is>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="G11" s="5" t="n">
         <v>43000</v>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="H11" s="5" t="n">
         <v>4800</v>
       </c>
-      <c r="H11" s="4" t="inlineStr"/>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr"/>
+      <c r="J11" s="4" t="inlineStr">
         <is>
           <t>약 4,800억원 (약 4억 3,000만 달러)</t>
         </is>
@@ -908,22 +959,27 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>VEM(터키)</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
+          <t>VEM</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>터키</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>빈혈치료제 바이오시밀러 생산기술</t>
         </is>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="G12" s="5" t="n">
         <v>300</v>
       </c>
-      <c r="G12" s="5" t="n">
+      <c r="H12" s="5" t="n">
         <v>33.4</v>
       </c>
-      <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="inlineStr">
         <is>
           <t>약 33억 4,000만원 (약 300만 달러)</t>
         </is>
@@ -945,24 +1001,29 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>익수다테라퓨틱스(영국)</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
+          <t>익수다테라퓨틱스</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>영국</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>항체약물접합체 플랫폼기술</t>
         </is>
       </c>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n">
+      <c r="G13" s="5" t="n"/>
+      <c r="H13" s="5" t="n">
         <v>4237</v>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>달러 금액 미표기</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>4,237억원</t>
         </is>
@@ -982,26 +1043,27 @@
           <t>대웅제약</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>중남미 4개국</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>위식도역류질환 치료제 '펙수프라잔(Fexuprazan)'</t>
         </is>
       </c>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n">
+      <c r="G14" s="5" t="n"/>
+      <c r="H14" s="5" t="n">
         <v>340</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>달러 금액 미표기</t>
-        </is>
-      </c>
       <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>원문에 상대사 미기재(수출 대상국만 표기), 달러 금액 미표기</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>약 340억원</t>
         </is>
@@ -1023,18 +1085,23 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>뤄신(중국)</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
+          <t>뤄신</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>'케이캡' 위식도 역류질환 치료주사</t>
         </is>
       </c>
-      <c r="F15" s="5" t="n"/>
       <c r="G15" s="5" t="n"/>
-      <c r="H15" s="4" t="inlineStr"/>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="H15" s="5" t="n"/>
+      <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>비공개</t>
         </is>
@@ -1056,24 +1123,29 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>카세릭스(호주)</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
+          <t>카세릭스</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>호주</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>CAR-T 치료제</t>
         </is>
       </c>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n">
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>달러 금액 미표기</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="J16" s="4" t="inlineStr">
         <is>
           <t>약 1,500억원</t>
         </is>
@@ -1095,24 +1167,29 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>피에르파브르(프랑스)</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
+          <t>피에르파브르</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>프랑스</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>고형암 치료를 위한 신규 항체 후보물질</t>
         </is>
       </c>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n">
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="5" t="n">
         <v>1164</v>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>달러 금액 미표기</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="J17" s="4" t="inlineStr">
         <is>
           <t>약 1,164억원</t>
         </is>
@@ -1134,22 +1211,31 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>인타스(다국적제약사)</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
+          <t>인타스</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>다국적</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>스텔라라 바이오시밀러 'DMB-3115'의 글로벌 라이선스 아웃 계약</t>
         </is>
       </c>
-      <c r="F18" s="5" t="n">
+      <c r="G18" s="5" t="n">
         <v>10500</v>
       </c>
-      <c r="G18" s="5" t="n">
+      <c r="H18" s="5" t="n">
         <v>1200</v>
       </c>
-      <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>원문 국가 표기는 '다국적제약사'</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
         <is>
           <t>약 1,200억원 (총 1억 500만 달러)</t>
         </is>
@@ -1171,18 +1257,23 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>양쯔강약업그룹(중국)</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
+          <t>양쯔강약업그룹</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>DA-7310(요로감염증)</t>
         </is>
       </c>
-      <c r="F19" s="5" t="n"/>
       <c r="G19" s="5" t="n"/>
-      <c r="H19" s="4" t="inlineStr"/>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="H19" s="5" t="n"/>
+      <c r="I19" s="4" t="inlineStr"/>
+      <c r="J19" s="4" t="inlineStr">
         <is>
           <t>비공개</t>
         </is>
@@ -1204,22 +1295,27 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>경신제약(중국)</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
+          <t>경신제약</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>소아연축·뇌전증 치료물질 계약</t>
         </is>
       </c>
-      <c r="F20" s="5" t="n">
+      <c r="G20" s="5" t="n">
         <v>4000</v>
       </c>
-      <c r="G20" s="5" t="n">
+      <c r="H20" s="5" t="n">
         <v>468</v>
       </c>
-      <c r="H20" s="4" t="inlineStr"/>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="I20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="inlineStr">
         <is>
           <t>468억원 (약 4,000만 달러)</t>
         </is>
@@ -1241,22 +1337,27 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>브리켈바이오텍(미국)</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
+          <t>브리켈바이오텍</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>미국</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>자가면역질환 치료제 프로그램</t>
         </is>
       </c>
-      <c r="F21" s="5" t="n">
+      <c r="G21" s="5" t="n">
         <v>32350</v>
       </c>
-      <c r="G21" s="5" t="n">
+      <c r="H21" s="5" t="n">
         <v>3800</v>
       </c>
-      <c r="H21" s="4" t="inlineStr"/>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="I21" s="4" t="inlineStr"/>
+      <c r="J21" s="4" t="inlineStr">
         <is>
           <t>약 3,800억원 (3억 2,350만 달러)</t>
         </is>
@@ -1278,26 +1379,31 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>선전 살루브리스 제약(중국)</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
+          <t>선전 살루브리스 제약</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>대사성질환 치료제 DD01</t>
         </is>
       </c>
-      <c r="F22" s="5" t="n">
+      <c r="G22" s="5" t="n">
         <v>400</v>
       </c>
-      <c r="G22" s="5" t="n">
+      <c r="H22" s="5" t="n">
         <v>47</v>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>총 계약규모 비공개, 계약금만 공개</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="J22" s="4" t="inlineStr">
         <is>
           <t>비공개 / 계약금 약 47억원 (약 400만 달러)</t>
         </is>
@@ -1319,22 +1425,27 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>한소제약(중국)</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
+          <t>한소제약</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>GalNAc-asiRNA 기반 기술 관련 신약후보물질 2종</t>
         </is>
       </c>
-      <c r="F23" s="5" t="n">
+      <c r="G23" s="5" t="n">
         <v>45100</v>
       </c>
-      <c r="G23" s="5" t="n">
+      <c r="H23" s="5" t="n">
         <v>5368</v>
       </c>
-      <c r="H23" s="4" t="inlineStr"/>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="I23" s="4" t="inlineStr"/>
+      <c r="J23" s="4" t="inlineStr">
         <is>
           <t>5,368억원 (약 4억 5,100만 달러)</t>
         </is>
@@ -1356,22 +1467,27 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>룬드벡(덴마크)</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
+          <t>룬드벡</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>덴마크</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>자가면역 질환 치료 후보물질 APB-A1</t>
         </is>
       </c>
-      <c r="F24" s="5" t="n">
+      <c r="G24" s="5" t="n">
         <v>44800</v>
       </c>
-      <c r="G24" s="5" t="n">
+      <c r="H24" s="5" t="n">
         <v>5370</v>
       </c>
-      <c r="H24" s="4" t="inlineStr"/>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="I24" s="4" t="inlineStr"/>
+      <c r="J24" s="4" t="inlineStr">
         <is>
           <t>약 5,370억원 (4억 4,800만 달러)</t>
         </is>
@@ -1393,22 +1509,31 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>아그라스(아랍에미리트) 등 중동 6개국(사우디아라비아·아랍에미리트·쿠웨이트·바레인·오만·카타르)</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
+          <t>아그라스 등</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>중동 6개국(사우디아라비아·아랍에미리트·쿠웨이트·바레인·오만·카타르)</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>위식도역류질환 치료 신약 '펙수프라잔' 라이선스아웃(기술수출)</t>
         </is>
       </c>
-      <c r="F25" s="5" t="n">
+      <c r="G25" s="5" t="n">
         <v>8466</v>
       </c>
-      <c r="G25" s="5" t="n">
+      <c r="H25" s="5" t="n">
         <v>991</v>
       </c>
-      <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>아그라스는 아랍에미리트 소재</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
         <is>
           <t>약 991억원 (약 8,466만 달러)</t>
         </is>
@@ -1430,22 +1555,27 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>테아오픈이노베이션(프랑스)</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
+          <t>테아오픈이노베이션</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>프랑스</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>당뇨병성 황반부종 및 습성 황반변성 치료제 'CU06-RE'</t>
         </is>
       </c>
-      <c r="F26" s="5" t="n">
+      <c r="G26" s="5" t="n">
         <v>16350</v>
       </c>
-      <c r="G26" s="5" t="n">
+      <c r="H26" s="5" t="n">
         <v>1906.9005</v>
       </c>
-      <c r="H26" s="4" t="inlineStr"/>
-      <c r="I26" s="4" t="inlineStr">
+      <c r="I26" s="4" t="inlineStr"/>
+      <c r="J26" s="4" t="inlineStr">
         <is>
           <t>약 1,906억 9,005만원 (1억 6,350만 달러)</t>
         </is>
@@ -1467,22 +1597,27 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>상해의약그룹 자회사 신이(중국)</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
+          <t>상해의약그룹 자회사 신이</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>면역질환 치료 소재 KBL697와 KBL693</t>
         </is>
       </c>
-      <c r="F27" s="5" t="n">
+      <c r="G27" s="5" t="n">
         <v>11000</v>
       </c>
-      <c r="G27" s="5" t="n">
+      <c r="H27" s="5" t="n">
         <v>1200</v>
       </c>
-      <c r="H27" s="4" t="inlineStr"/>
-      <c r="I27" s="4" t="inlineStr">
+      <c r="I27" s="4" t="inlineStr"/>
+      <c r="J27" s="4" t="inlineStr">
         <is>
           <t>약 1,200억원 (1억 1,000만 달러)</t>
         </is>
@@ -1504,22 +1639,27 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>앱토즈 바이오사이언스(캐나다)</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
+          <t>앱토즈 바이오사이언스</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>캐나다</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>급성골수성 백혈병(AML) 치료 신약 'HM43239'</t>
         </is>
       </c>
-      <c r="F28" s="5" t="n">
+      <c r="G28" s="5" t="n">
         <v>42000</v>
       </c>
-      <c r="G28" s="5" t="n">
+      <c r="H28" s="5" t="n">
         <v>4961</v>
       </c>
-      <c r="H28" s="4" t="inlineStr"/>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="I28" s="4" t="inlineStr"/>
+      <c r="J28" s="4" t="inlineStr">
         <is>
           <t>약 4,961억원 (4억 2,000만 달러)</t>
         </is>
@@ -1541,26 +1681,31 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>이그니스테라퓨틱스(중국)</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
+          <t>이그니스테라퓨틱스</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>세노바메이트 등 6개 CNS 신약</t>
         </is>
       </c>
-      <c r="F29" s="5" t="n">
+      <c r="G29" s="5" t="n">
         <v>18500</v>
       </c>
-      <c r="G29" s="5" t="n">
+      <c r="H29" s="5" t="n">
         <v>2180</v>
       </c>
-      <c r="H29" s="4" t="inlineStr">
+      <c r="I29" s="4" t="inlineStr">
         <is>
           <t>지분 형태</t>
         </is>
       </c>
-      <c r="I29" s="4" t="inlineStr">
+      <c r="J29" s="4" t="inlineStr">
         <is>
           <t>약 2,180억원(지분) (1억 8,500만 달러)</t>
         </is>
@@ -1582,22 +1727,27 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>피라미드바이오사이언스(미국)</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
+          <t>피라미드바이오사이언스</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>미국</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>MPS1 타겟 고형암치료제(VRN08)</t>
         </is>
       </c>
-      <c r="F30" s="5" t="n">
+      <c r="G30" s="5" t="n">
         <v>84600</v>
       </c>
-      <c r="G30" s="5" t="n">
+      <c r="H30" s="5" t="n">
         <v>10000</v>
       </c>
-      <c r="H30" s="4" t="inlineStr"/>
-      <c r="I30" s="4" t="inlineStr">
+      <c r="I30" s="4" t="inlineStr"/>
+      <c r="J30" s="4" t="inlineStr">
         <is>
           <t>약 1조원 (8억 4,600만 달러)</t>
         </is>
@@ -1619,22 +1769,27 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>소티오바이오텍(체코)</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
+          <t>소티오바이오텍</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>체코</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>항체약물접합체(ADC) 플랫폼 기술</t>
         </is>
       </c>
-      <c r="F31" s="5" t="n">
+      <c r="G31" s="5" t="n">
         <v>102750</v>
       </c>
-      <c r="G31" s="5" t="n">
+      <c r="H31" s="5" t="n">
         <v>12127</v>
       </c>
-      <c r="H31" s="4" t="inlineStr"/>
-      <c r="I31" s="4" t="inlineStr">
+      <c r="I31" s="4" t="inlineStr"/>
+      <c r="J31" s="4" t="inlineStr">
         <is>
           <t>약 1조 2,127억원 (10억 2,750만 달러)</t>
         </is>
@@ -1656,22 +1811,27 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>엔도그룹(아일랜드)</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
+          <t>엔도그룹</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>아일랜드</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>세노바메이트</t>
         </is>
       </c>
-      <c r="F32" s="5" t="n">
+      <c r="G32" s="5" t="n">
         <v>4100</v>
       </c>
-      <c r="G32" s="5" t="n">
+      <c r="H32" s="5" t="n">
         <v>433.0465</v>
       </c>
-      <c r="H32" s="4" t="inlineStr"/>
-      <c r="I32" s="4" t="inlineStr">
+      <c r="I32" s="4" t="inlineStr"/>
+      <c r="J32" s="4" t="inlineStr">
         <is>
           <t>433억 465만원 / 4,100만 달러</t>
         </is>
@@ -1693,22 +1853,27 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>브레인트리 래보라토리스(미국)</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
+          <t>브레인트리 래보라토리스</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>미국</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
         <is>
           <t>케이캡(테고프라잔)</t>
         </is>
       </c>
-      <c r="F33" s="5" t="n">
+      <c r="G33" s="5" t="n">
         <v>54000</v>
       </c>
-      <c r="G33" s="5" t="n">
+      <c r="H33" s="5" t="n">
         <v>6400</v>
       </c>
-      <c r="H33" s="4" t="inlineStr"/>
-      <c r="I33" s="4" t="inlineStr">
+      <c r="I33" s="4" t="inlineStr"/>
+      <c r="J33" s="4" t="inlineStr">
         <is>
           <t>6,400억원 / 5억 4,000만 달러</t>
         </is>
@@ -1730,22 +1895,27 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>익수다테라퓨틱스(영국)</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
+          <t>익수다테라퓨틱스</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>영국</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>표적유방암치료제 LCB14(HER2-ADC)</t>
         </is>
       </c>
-      <c r="F34" s="5" t="n">
+      <c r="G34" s="5" t="n">
         <v>100000</v>
       </c>
-      <c r="G34" s="5" t="n">
+      <c r="H34" s="5" t="n">
         <v>11864</v>
       </c>
-      <c r="H34" s="4" t="inlineStr"/>
-      <c r="I34" s="4" t="inlineStr">
+      <c r="I34" s="4" t="inlineStr"/>
+      <c r="J34" s="4" t="inlineStr">
         <is>
           <t>1조 1,864억원 / 10억 달러</t>
         </is>
@@ -1767,22 +1937,27 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>에퍼메드 테라퓨틱스(중국)</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
+          <t>에퍼메드 테라퓨틱스</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>안과분야 신약 루미네이트(리수테가닙)</t>
         </is>
       </c>
-      <c r="F35" s="5" t="n">
+      <c r="G35" s="5" t="n">
         <v>14500</v>
       </c>
-      <c r="G35" s="5" t="n">
+      <c r="H35" s="5" t="n">
         <v>1719</v>
       </c>
-      <c r="H35" s="4" t="inlineStr"/>
-      <c r="I35" s="4" t="inlineStr">
+      <c r="I35" s="4" t="inlineStr"/>
+      <c r="J35" s="4" t="inlineStr">
         <is>
           <t>약 1,719억원 / 1억 4,500만 달러</t>
         </is>
@@ -1801,20 +1976,21 @@
       <c r="C36" s="7" t="n"/>
       <c r="D36" s="7" t="n"/>
       <c r="E36" s="7" t="n"/>
-      <c r="F36" s="8">
-        <f>SUM(F3:F35)</f>
-        <v/>
-      </c>
+      <c r="F36" s="7" t="n"/>
       <c r="G36" s="8">
         <f>SUM(G3:G35)</f>
         <v/>
       </c>
-      <c r="H36" s="9" t="inlineStr">
+      <c r="H36" s="8">
+        <f>SUM(H3:H35)</f>
+        <v/>
+      </c>
+      <c r="I36" s="9" t="inlineStr">
         <is>
           <t>비공개 건 제외 합계</t>
         </is>
       </c>
-      <c r="I36" s="7" t="n"/>
+      <c r="J36" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
@@ -1826,28 +2002,35 @@
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>※ 원문 표에는 달러 금액이 없는 건이 있어 '계약규모(만달러)' 합계 건수는 '계약규모(억원)' 합계 건수보다 적음.</t>
+          <t>※ 원문 표의 '계약상대(국가)' 한 칸을 계약상대 / 국가 두 열로 분리함.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>※ 원문 표기 총액은 13조 3,720억원. 본 시트의 억원 합계는 원문 각 행을 반올림 없이 더한 값이라 약 13억원(0.01%) 차이가 남.</t>
+          <t>※ 원문 표에는 달러 금액이 없는 건이 있어 '계약규모(만달러)' 합계 건수는 '계약규모(억원)' 합계 건수보다 적음.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
         <is>
+          <t>※ 원문 표기 총액은 13조 3,720억원. 본 시트의 억원 합계는 원문 각 행을 반올림 없이 더한 값이라 약 13억원(0.01%) 차이가 남.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
           <t>※ 원문 표에 연도 표기가 없음(일자 1. 7. ~ 12. 31. 1년치).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:I35"/>
+  <autoFilter ref="A2:J35"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>